<commit_message>
Complete DeepWeeds submission report and result tables
</commit_message>
<xml_diff>
--- a/submissions/2026A02939_TranCaoQuocDinh/results.xlsx
+++ b/submissions/2026A02939_TranCaoQuocDinh/results.xlsx
@@ -17,11 +17,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$M$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$Q$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PerClass'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Latency'!$A$1:$N$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$P$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$N$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PerClass'!$A$1:$G$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Latency'!$A$1:$O$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -771,7 +771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -781,7 +781,7 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
@@ -883,37 +883,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>convnext_tiny</t>
+          <t>resnet50</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8656963341817592</v>
+        <v>0.8712313173670629</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8908883176235362</v>
+        <v>0.9031705227077977</v>
       </c>
       <c r="F2" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G2" t="n">
-        <v>27.827049</v>
-      </c>
-      <c r="H2" t="inlineStr"/>
+        <v>23.526473</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.131713024</v>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
-        <v>93.66681196083334</v>
+        <v>110.8720678005833</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>frozen</t>
+          <t>finetune</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -930,39 +932,41 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>-0.1018231164925144</v>
+        <v>-0.09628813330721064</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>convnext_tiny</t>
+          <t>resnet50</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9632944132792739</v>
+        <v>0.8575700883639924</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9700085689802913</v>
+        <v>0.8946015424164524</v>
       </c>
       <c r="F3" t="n">
         <v>11</v>
       </c>
       <c r="G3" t="n">
-        <v>27.827049</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
+        <v>23.526473</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.131713024</v>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>252.5959650525834</v>
+        <v>113.9269334256667</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -971,7 +975,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>color</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -983,39 +987,41 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>-0.004225037394999687</v>
+        <v>-0.1099493623102812</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>convnext_tiny</t>
+          <t>resnet50</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>0.961665075767857</v>
+        <v>0.8525651798842351</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9700085689802913</v>
+        <v>0.8903170522707797</v>
       </c>
       <c r="F4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G4" t="n">
-        <v>27.827049</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
+        <v>23.526473</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4.131713024</v>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
-        <v>159.8644468082502</v>
+        <v>133.8305945927503</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1024,7 +1030,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>randaug</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1036,13 +1042,13 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>-0.005854374906416604</v>
+        <v>-0.1149542707900385</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1054,13 +1060,13 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9614439386240947</v>
+        <v>0.8656963341817592</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9714367323621822</v>
+        <v>0.8908883176235362</v>
       </c>
       <c r="F5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
         <v>27.827049</v>
@@ -1068,11 +1074,11 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>161.1655075020832</v>
+        <v>93.66681196083334</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>finetune</t>
+          <t>frozen</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1082,20 +1088,20 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ls</t>
+          <t>ce</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>-0.006075512050178866</v>
+        <v>-0.1018231164925144</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1107,13 +1113,13 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9645034007962335</v>
+        <v>0.9632944132792739</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9717223650385605</v>
+        <v>0.9700085689802913</v>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G6" t="n">
         <v>27.827049</v>
@@ -1121,7 +1127,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
-        <v>135.3420451692502</v>
+        <v>252.5959650525834</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1130,25 +1136,25 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>color</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>focal</t>
+          <t>ce</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>-0.00301604987804005</v>
+        <v>-0.004225037394999687</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1160,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9610835820742208</v>
+        <v>0.961665075767857</v>
       </c>
       <c r="E7" t="n">
         <v>0.9700085689802913</v>
       </c>
       <c r="F7" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
         <v>27.827049</v>
@@ -1174,7 +1180,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
-        <v>131.4183403762504</v>
+        <v>159.8644468082502</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1183,25 +1189,25 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>randaug</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ce_weighted</t>
+          <t>ce</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>-0.006435868600052741</v>
+        <v>-0.005854374906416604</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1213,13 +1219,13 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9550207986181307</v>
+        <v>0.9614439386240947</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9642959154527277</v>
+        <v>0.9714367323621822</v>
       </c>
       <c r="F8" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G8" t="n">
         <v>27.827049</v>
@@ -1227,7 +1233,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
-        <v>223.3140612997501</v>
+        <v>161.1655075020832</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1236,23 +1242,182 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>color</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>focal</t>
+          <t>ls</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
+        <v>-0.006075512050178866</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.9645034007962335</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9717223650385605</v>
+      </c>
+      <c r="F9" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>135.3420451692502</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>finetune</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>focal</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="n">
+        <v>-0.00301604987804005</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9610835820742208</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9700085689802913</v>
+      </c>
+      <c r="F10" t="n">
+        <v>11</v>
+      </c>
+      <c r="G10" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>131.4183403762504</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>finetune</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>ce_weighted</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="n">
+        <v>-0.006435868600052741</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.9550207986181307</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9642959154527277</v>
+      </c>
+      <c r="F11" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>223.3140612997501</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>finetune</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>focal</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="n">
         <v>-0.01249865205614287</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q8"/>
+  <autoFilter ref="A1:Q11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1263,10 +1428,401 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <autoFilter ref="A1:A1"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>exp_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1_val</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>top1_val</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ece_val</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>p50_ms</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>p95_ms</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>p99_ms</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>images_per_s</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>relative_p50</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>gpu</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>dtype</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>preprocessing_included</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>I00_one_view</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9675194506742736</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9745786918023421</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.01645694729669614</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5.988715999933447</v>
+      </c>
+      <c r="I2" t="n">
+        <v>9.384225549945313</v>
+      </c>
+      <c r="J2" t="n">
+        <v>9.485997240001325</v>
+      </c>
+      <c r="K2" t="n">
+        <v>166.9807017081981</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>I01_hflip</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.967661915407397</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9748643244787204</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.01435841474829998</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>11.43984850000379</v>
+      </c>
+      <c r="I3" t="n">
+        <v>12.04195675006758</v>
+      </c>
+      <c r="J3" t="n">
+        <v>13.2008403400664</v>
+      </c>
+      <c r="K3" t="n">
+        <v>87.4137450333952</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1.91023392996611</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>I02_five_crop_prob</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9683727505759845</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9754355898314767</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.01284442184414742</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>31.37005199994292</v>
+      </c>
+      <c r="I4" t="n">
+        <v>32.61622495000438</v>
+      </c>
+      <c r="J4" t="n">
+        <v>34.64449641008514</v>
+      </c>
+      <c r="K4" t="n">
+        <v>31.87753721293862</v>
+      </c>
+      <c r="L4" t="n">
+        <v>5.23819329557313</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>I03_five_crop_logit</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9683727505759845</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9754355898314767</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.01360889603600643</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>31.37005199994292</v>
+      </c>
+      <c r="I5" t="n">
+        <v>32.61622495000438</v>
+      </c>
+      <c r="J5" t="n">
+        <v>34.64449641008514</v>
+      </c>
+      <c r="K5" t="n">
+        <v>31.87753721293862</v>
+      </c>
+      <c r="L5" t="n">
+        <v>5.23819329557313</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>I04_temperature</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.9675194506742736</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9745786918023421</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.007525448749826508</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5.988715999933447</v>
+      </c>
+      <c r="I6" t="n">
+        <v>9.384225549945313</v>
+      </c>
+      <c r="J6" t="n">
+        <v>9.485997240001325</v>
+      </c>
+      <c r="K6" t="n">
+        <v>166.9807017081981</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1277,10 +1833,467 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <autoFilter ref="A1:A1"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>exp_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>backbone</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1_val</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>top1_val</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>best_epoch</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>params_m</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>gmac</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>latency_batch1_ms</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>train_seconds_per_epoch</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1_test</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>top1_test</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ece_test</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>inference_method</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9675194506742736</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9745786918023421</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G2" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.454808576</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="n">
+        <v>134.1112931853334</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.9698884328006913</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.9754776161961791</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.01176129059024804</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>I02_five_crop_prob</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.9672955482454922</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9748643244787204</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.454808576</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>124.0938747689167</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.9681397733012257</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.9754776161961791</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.01170832150841179</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>I02_five_crop_prob</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9622818627320819</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9697229363039132</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G4" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4.454808576</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>209.6579149323331</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.9640123338854547</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.9717707442258341</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.01211785852010269</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>I02_five_crop_prob</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.8712313173670629</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9031705227077977</v>
+      </c>
+      <c r="F5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G5" t="n">
+        <v>23.526473</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4.131713024</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>110.8720678005833</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.8742436997257693</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.9019104647847163</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.01362621563444533</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>I00_one_view</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8575700883639924</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.8946015424164524</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" t="n">
+        <v>23.526473</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4.131713024</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>113.9269334256667</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.8606923213896429</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.8950670088394639</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.01828233169945824</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>I00_one_view</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.8525651798842351</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.8903170522707797</v>
+      </c>
+      <c r="F7" t="n">
+        <v>11</v>
+      </c>
+      <c r="G7" t="n">
+        <v>23.526473</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4.131713024</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>133.8305945927503</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.8620758053513703</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.8933561448531508</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.01648715500712871</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>I00_one_view</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.9657 +/- 0.0030</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0.9673 +/- 0.0030</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0.9742 +/- 0.0021</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0.0119 +/- 0.0002</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.8605 +/- 0.0097</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0.8657 +/- 0.0075</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0.8968 +/- 0.0045</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>0.0161 +/- 0.0023</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1291,10 +2304,2145 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <autoFilter ref="A1:A1"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>exp_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>precision</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Chinee Apple</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>226</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9727272727272728</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.9469026548672567</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.9596412556053813</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>213</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9812206572769953</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.9653579676674364</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>207</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9900990099009901</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.966183574879227</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.9779951100244499</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>205</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9609756097560975</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9728395061728395</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Prickly Acacia</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>213</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9251101321585903</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.9859154929577465</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.9545454545454545</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Rubber Vine</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>202</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.9847715736040609</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.9603960396039604</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.9724310776942354</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Siam Weed</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>215</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9813953488372092</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.9813953488372092</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.9813953488372092</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Snake Weed</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>204</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9796954314720813</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.946078431372549</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.9625935162094763</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Negatives</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1822</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9803171131765992</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.9840834248079035</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.9821966584497398</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Chinee Apple</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>226</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9678899082568807</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.9336283185840708</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.9504504504504504</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>213</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.9541284403669725</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.9765258215962441</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.9651972157772623</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>207</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.9577464788732394</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.9855072463768116</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.9714285714285714</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>205</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.9710144927536232</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.9804878048780488</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.9757281553398058</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Prickly Acacia</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>213</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.9403669724770642</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.9624413145539906</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.9512761020881672</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Rubber Vine</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>202</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.9801980198019802</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.9801980198019802</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.9801980198019802</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Siam Weed</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>215</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.9724770642201835</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.986046511627907</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.979214780600462</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Snake Weed</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>204</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.946078431372549</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.9554455445544553</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Negatives</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1822</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.9867622724765582</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.9818880351262349</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.9843191196698762</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Chinee Apple</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>226</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.9813953488372092</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.9336283185840708</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.9569160997732425</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>213</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.9669811320754716</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.9624413145539906</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.9647058823529412</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>207</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.9759615384615384</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.9806763285024155</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.9783132530120482</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>205</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.9747474747474747</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.9414634146341463</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.9578163771712158</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Prickly Acacia</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>213</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.9151785714285714</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.9624413145539906</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.9382151029748282</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Rubber Vine</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>202</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.9898477157360406</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.9653465346534653</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.9774436090225563</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Siam Weed</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>215</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.9636363636363636</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.986046511627907</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.974712643678161</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Snake Weed</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>204</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.9740932642487047</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.9215686274509803</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.947103274559194</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Negatives</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1822</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.9760869565217392</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.9857299670691547</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.9808847624249044</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Chinee Apple</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>226</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.9041916167664671</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.668141592920354</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.7684478371501272</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>213</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.8434782608695652</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.9107981220657277</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.8758465011286682</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>207</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.9216589861751152</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.966183574879227</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.9433962264150944</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>205</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.9580838323353293</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.7804878048780488</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.860215053763441</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Prickly Acacia</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>213</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.7950819672131147</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.9107981220657277</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.849015317286652</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Rubber Vine</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>202</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.9459459459459459</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.8663366336633663</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.9043927648578812</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Siam Weed</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>215</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.8930232558139535</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.9164677804295943</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Snake Weed</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>204</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.8813559322033898</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.7647058823529411</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.8188976377952756</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Negatives</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1822</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.9086638830897703</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.955543358946213</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.9315141787051899</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Chinee Apple</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>226</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.5575221238938053</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.6980609418282548</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>213</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.8995215311004785</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.8826291079812206</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.8909952606635071</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>207</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.90625</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.9806763285024155</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.9419953596287703</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>205</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.9440993788819876</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.7414634146341463</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.8306010928961749</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Prickly Acacia</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>213</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.8409090909090909</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.8685446009389671</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.8545034642032332</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Rubber Vine</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>202</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.9497206703910615</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.8415841584158416</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.8923884514435696</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Siam Weed</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>215</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.8868778280542986</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.9116279069767442</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.8990825688073395</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Snake Weed</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>204</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.837696335078534</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.7843137254901961</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.810126582278481</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Negatives</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1822</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.8942552109811897</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.9654226125137212</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.9284771707574558</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Chinee Apple</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>226</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.9710144927536232</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.5929203539823009</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.7362637362637363</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>213</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.8970588235294118</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.8591549295774648</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.8776978417266187</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>207</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.9220183486238532</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.9710144927536232</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.9458823529411765</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>205</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.9487179487179487</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.7219512195121951</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.8199445983379502</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Prickly Acacia</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>213</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.8502415458937198</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.8262910798122066</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.8380952380952381</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Rubber Vine</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>202</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.9086294416243654</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.8861386138613861</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.8972431077694236</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Siam Weed</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>215</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.8717948717948718</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.9488372093023256</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.9086859688195991</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Snake Weed</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>204</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.884393063583815</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.8116710875331565</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Negatives</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>1822</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.8863636363636364</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.9632272228320526</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.9231983166754339</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Chinee Apple</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>226</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0.9740 +/- 0.0068</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>0.9381 +/- 0.0077</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>0.9557 +/- 0.0047</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>213</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>0.9570 +/- 0.0089</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>0.9734 +/- 0.0098</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>0.9651 +/- 0.0003</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Negatives</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1822</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>0.9811 +/- 0.0054</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>0.9839 +/- 0.0019</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>0.9825 +/- 0.0017</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>207</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0.9746 +/- 0.0162</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>0.9775 +/- 0.0101</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>0.9759 +/- 0.0039</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>205</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>0.9769 +/- 0.0072</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>0.9610 +/- 0.0195</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>0.9688 +/- 0.0096</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Prickly Acacia</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>213</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>0.9269 +/- 0.0127</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>0.9703 +/- 0.0136</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>0.9480 +/- 0.0086</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Rubber Vine</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>202</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>0.9849 +/- 0.0048</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>0.9686 +/- 0.0103</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>0.9767 +/- 0.0039</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Siam Weed</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>215</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>0.9725 +/- 0.0089</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>0.9845 +/- 0.0027</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>0.9784 +/- 0.0034</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Snake Weed</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>204</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>0.9729 +/- 0.0074</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>0.9379 +/- 0.0142</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>0.9550 +/- 0.0078</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Chinee Apple</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>226</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>0.9362 +/- 0.0335</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>0.6062 +/- 0.0565</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>0.7343 +/- 0.0352</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>213</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>0.8800 +/- 0.0317</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>0.8842 +/- 0.0259</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>0.8815 +/- 0.0083</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Negatives</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1822</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>0.8964 +/- 0.0113</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>0.9614 +/- 0.0052</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>0.9277 +/- 0.0042</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>207</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>0.9166 +/- 0.0090</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>0.9726 +/- 0.0074</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>0.9438 +/- 0.0020</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>205</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>0.9503 +/- 0.0071</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>0.7480 +/- 0.0298</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>0.8369 +/- 0.0209</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Prickly Acacia</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>213</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>0.8287 +/- 0.0295</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>0.8685 +/- 0.0423</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>0.8472 +/- 0.0084</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Rubber Vine</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>202</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>0.9348 +/- 0.0227</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>0.8647 +/- 0.0223</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>0.8980 +/- 0.0060</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Siam Weed</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>215</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>0.8999 +/- 0.0365</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>0.9178 +/- 0.0284</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>0.9081 +/- 0.0087</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>mean +/- std</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Snake Weed</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>204</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>0.8678 +/- 0.0261</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>0.7663 +/- 0.0172</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>0.8136 +/- 0.0047</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1305,16 +4453,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -1322,6 +4470,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1395,6 +4544,11 @@
           <t>torch</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>k_views</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1449,6 +4603,7 @@
           <t>2.11.0+cu128</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1503,6 +4658,7 @@
           <t>2.11.0+cu128</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1557,6 +4713,7 @@
           <t>2.11.0+cu128</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1611,6 +4768,7 @@
           <t>2.11.0+cu128</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1665,9 +4823,291 @@
           <t>2.11.0+cu128</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>I00_one_view</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5.988715999933447</v>
+      </c>
+      <c r="E7" t="n">
+        <v>9.384225549945313</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9.485997240001325</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6.402375960001336</v>
+      </c>
+      <c r="H7" t="n">
+        <v>50</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>224</v>
+      </c>
+      <c r="M7" t="n">
+        <v>166.9807017081981</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>I01_hflip</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>11.43984850000379</v>
+      </c>
+      <c r="E8" t="n">
+        <v>12.04195675006758</v>
+      </c>
+      <c r="F8" t="n">
+        <v>13.2008403400664</v>
+      </c>
+      <c r="G8" t="n">
+        <v>11.4937040399991</v>
+      </c>
+      <c r="H8" t="n">
+        <v>50</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>224</v>
+      </c>
+      <c r="M8" t="n">
+        <v>87.4137450333952</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>I02_five_crop_prob</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>31.37005199994292</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32.61622495000438</v>
+      </c>
+      <c r="F9" t="n">
+        <v>34.64449641008514</v>
+      </c>
+      <c r="G9" t="n">
+        <v>31.51935257999867</v>
+      </c>
+      <c r="H9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>224</v>
+      </c>
+      <c r="M9" t="n">
+        <v>31.87753721293862</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>I03_five_crop_logit</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>31.37005199994292</v>
+      </c>
+      <c r="E10" t="n">
+        <v>32.61622495000438</v>
+      </c>
+      <c r="F10" t="n">
+        <v>34.64449641008514</v>
+      </c>
+      <c r="G10" t="n">
+        <v>31.51935257999867</v>
+      </c>
+      <c r="H10" t="n">
+        <v>50</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>224</v>
+      </c>
+      <c r="M10" t="n">
+        <v>31.87753721293862</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>I04_temperature</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5.988715999933447</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9.384225549945313</v>
+      </c>
+      <c r="F11" t="n">
+        <v>9.485997240001325</v>
+      </c>
+      <c r="G11" t="n">
+        <v>6.402375960001336</v>
+      </c>
+      <c r="H11" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>224</v>
+      </c>
+      <c r="M11" t="n">
+        <v>166.9807017081981</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N6"/>
+  <autoFilter ref="A1:O11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1682,14 +5122,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
@@ -1793,7 +5233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1805,30 +5245,32 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9645034007962335</v>
+        <v>0.9675194506742736</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9717223650385605</v>
+        <v>0.9745786918023421</v>
       </c>
       <c r="F3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" t="n">
         <v>27.827049</v>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>4.454808576</v>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>135.3420451692502</v>
+        <v>134.1112931853334</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0129660721908026</v>
+        <v>0.01645702195372755</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1837,33 +5279,35 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9632944132792739</v>
+        <v>0.9672955482454922</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9700085689802913</v>
+        <v>0.9748643244787204</v>
       </c>
       <c r="F4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G4" t="n">
         <v>27.827049</v>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>4.454808576</v>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
-        <v>252.5959650525834</v>
+        <v>124.0938747689167</v>
       </c>
       <c r="K4" t="n">
-        <v>0.01946913129105969</v>
+        <v>0.0138350834047414</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1875,13 +5319,13 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.961665075767857</v>
+        <v>0.9645034007962335</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9700085689802913</v>
+        <v>0.9717223650385605</v>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
         <v>27.827049</v>
@@ -1889,16 +5333,16 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>159.8644468082502</v>
+        <v>135.3420451692502</v>
       </c>
       <c r="K5" t="n">
-        <v>0.01492908996858035</v>
+        <v>0.0129660721908026</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1910,10 +5354,10 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9614439386240947</v>
+        <v>0.9632944132792739</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9714367323621822</v>
+        <v>0.9700085689802913</v>
       </c>
       <c r="F6" t="n">
         <v>11</v>
@@ -1924,16 +5368,16 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
-        <v>161.1655075020832</v>
+        <v>252.5959650525834</v>
       </c>
       <c r="K6" t="n">
-        <v>0.07859627548700372</v>
+        <v>0.01946913129105969</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1942,33 +5386,35 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9610835820742208</v>
+        <v>0.9622818627320819</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9700085689802913</v>
+        <v>0.9697229363039132</v>
       </c>
       <c r="F7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G7" t="n">
         <v>27.827049</v>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>4.454808576</v>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
-        <v>131.4183403762504</v>
+        <v>209.6579149323331</v>
       </c>
       <c r="K7" t="n">
-        <v>0.01415334088546128</v>
+        <v>0.01834415041416737</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1980,13 +5426,13 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9550207986181307</v>
+        <v>0.961665075767857</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9642959154527277</v>
+        <v>0.9700085689802913</v>
       </c>
       <c r="F8" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G8" t="n">
         <v>27.827049</v>
@@ -1994,127 +5440,115 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
-        <v>223.3140612997501</v>
+        <v>159.8644468082502</v>
       </c>
       <c r="K8" t="n">
-        <v>0.01262933419308782</v>
+        <v>0.01492908996858035</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>vit_small_patch16_224</t>
+          <t>convnext_tiny</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9458499360621921</v>
+        <v>0.9614439386240947</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9597257926306769</v>
+        <v>0.9714367323621822</v>
       </c>
       <c r="F9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G9" t="n">
-        <v>21.669129</v>
-      </c>
-      <c r="H9" t="n">
-        <v>4.240838016</v>
-      </c>
-      <c r="I9" t="n">
-        <v>5.75501449930016</v>
-      </c>
+        <v>27.827049</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
-        <v>369.6720731578333</v>
+        <v>161.1655075020832</v>
       </c>
       <c r="K9" t="n">
-        <v>0.02119698950871177</v>
+        <v>0.07859627548700372</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>resnext50_32x4d</t>
+          <t>convnext_tiny</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8934738323413968</v>
+        <v>0.9610835820742208</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9180234218794631</v>
+        <v>0.9700085689802913</v>
       </c>
       <c r="F10" t="n">
         <v>11</v>
       </c>
       <c r="G10" t="n">
-        <v>22.998345</v>
-      </c>
-      <c r="H10" t="n">
-        <v>4.286154752</v>
-      </c>
-      <c r="I10" t="n">
-        <v>8.419552499617566</v>
-      </c>
+        <v>27.827049</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
-        <v>142.5327491406666</v>
+        <v>131.4183403762504</v>
       </c>
       <c r="K10" t="n">
-        <v>0.01952840829762918</v>
+        <v>0.01415334088546128</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B05</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>efficientnet_b0</t>
+          <t>convnext_tiny</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8746837328609423</v>
+        <v>0.9550207986181307</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9031705227077977</v>
+        <v>0.9642959154527277</v>
       </c>
       <c r="F11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G11" t="n">
-        <v>4.019077</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.384610272</v>
-      </c>
-      <c r="I11" t="n">
-        <v>8.12610550201498</v>
-      </c>
+        <v>27.827049</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>367.2788949341663</v>
+        <v>223.3140612997501</v>
       </c>
       <c r="K11" t="n">
-        <v>0.02830994199085975</v>
+        <v>0.01262933419308782</v>
       </c>
     </row>
   </sheetData>

</xml_diff>